<commit_message>
Otomatik veri güncelleme (06.08.2026 13:21 UTC)
</commit_message>
<xml_diff>
--- a/enflasyon/enflasyon.xlsx
+++ b/enflasyon/enflasyon.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E259"/>
+  <dimension ref="A1:E260"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4784,6 +4784,23 @@
       </c>
       <c r="E259" t="n">
         <v>17.75847125552932</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B260" t="n">
+        <v>132.31</v>
+      </c>
+      <c r="C260" t="n">
+        <v>1.784752673282552</v>
+      </c>
+      <c r="D260" t="n">
+        <v>31.75409679062435</v>
+      </c>
+      <c r="E260" t="n">
+        <v>19.86016871927905</v>
       </c>
     </row>
   </sheetData>
@@ -4797,7 +4814,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N259"/>
+  <dimension ref="A1:N260"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16222,6 +16239,50 @@
       </c>
       <c r="N259" t="n">
         <v>122.11</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B260" t="n">
+        <v>134.02</v>
+      </c>
+      <c r="C260" t="n">
+        <v>130.15</v>
+      </c>
+      <c r="D260" t="n">
+        <v>111.73</v>
+      </c>
+      <c r="E260" t="n">
+        <v>144.81</v>
+      </c>
+      <c r="F260" t="n">
+        <v>124.31</v>
+      </c>
+      <c r="G260" t="n">
+        <v>145.05</v>
+      </c>
+      <c r="H260" t="n">
+        <v>133.69</v>
+      </c>
+      <c r="I260" t="n">
+        <v>125.22</v>
+      </c>
+      <c r="J260" t="n">
+        <v>126.2</v>
+      </c>
+      <c r="K260" t="n">
+        <v>141.62</v>
+      </c>
+      <c r="L260" t="n">
+        <v>133.7</v>
+      </c>
+      <c r="M260" t="n">
+        <v>130.47</v>
+      </c>
+      <c r="N260" t="n">
+        <v>123.47</v>
       </c>
     </row>
   </sheetData>
@@ -16235,7 +16296,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N259"/>
+  <dimension ref="A1:N260"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27348,6 +27409,50 @@
       </c>
       <c r="N259" t="n">
         <v>22.71116817298007</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B260" t="n">
+        <v>37.53005127954092</v>
+      </c>
+      <c r="C260" t="n">
+        <v>29.38189201377268</v>
+      </c>
+      <c r="D260" t="n">
+        <v>16.47854628756089</v>
+      </c>
+      <c r="E260" t="n">
+        <v>40.32266749804405</v>
+      </c>
+      <c r="F260" t="n">
+        <v>22.40688250729537</v>
+      </c>
+      <c r="G260" t="n">
+        <v>43.89126368322292</v>
+      </c>
+      <c r="H260" t="n">
+        <v>30.83239164895124</v>
+      </c>
+      <c r="I260" t="n">
+        <v>23.96797719523978</v>
+      </c>
+      <c r="J260" t="n">
+        <v>23.35550153845947</v>
+      </c>
+      <c r="K260" t="n">
+        <v>44.18197132280049</v>
+      </c>
+      <c r="L260" t="n">
+        <v>31.65071076529042</v>
+      </c>
+      <c r="M260" t="n">
+        <v>25.64466844969539</v>
+      </c>
+      <c r="N260" t="n">
+        <v>21.73888482986941</v>
       </c>
     </row>
   </sheetData>
@@ -27408,16 +27513,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>131.89</v>
+        <v>134.02</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1670843776106823</v>
+        <v>1.614982182121483</v>
       </c>
       <c r="E2" t="n">
-        <v>35.44570668685729</v>
+        <v>37.53005127954092</v>
       </c>
       <c r="F2" t="n">
-        <v>19.89031433398294</v>
+        <v>21.82652154856619</v>
       </c>
     </row>
     <row r="3">
@@ -27432,16 +27537,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>127.68</v>
+        <v>130.15</v>
       </c>
       <c r="D3" t="n">
-        <v>3.460011344299496</v>
+        <v>1.934523809523814</v>
       </c>
       <c r="E3" t="n">
-        <v>34.15396359365354</v>
+        <v>29.38189201377268</v>
       </c>
       <c r="F3" t="n">
-        <v>14.07994837880906</v>
+        <v>16.2868521420896</v>
       </c>
     </row>
     <row r="4">
@@ -27456,16 +27561,16 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>116.3</v>
+        <v>111.73</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.1802420393099413</v>
+        <v>-3.929492691315561</v>
       </c>
       <c r="E4" t="n">
-        <v>14.18455344206522</v>
+        <v>16.47854628756089</v>
       </c>
       <c r="F4" t="n">
-        <v>6.961654984383214</v>
+        <v>2.758604569261713</v>
       </c>
     </row>
     <row r="5">
@@ -27480,16 +27585,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>141.62</v>
+        <v>144.81</v>
       </c>
       <c r="D5" t="n">
-        <v>2.297023981508239</v>
+        <v>2.252506708092072</v>
       </c>
       <c r="E5" t="n">
-        <v>45.14201960040407</v>
+        <v>40.32266749804405</v>
       </c>
       <c r="F5" t="n">
-        <v>23.14544261226892</v>
+        <v>25.91930196781995</v>
       </c>
     </row>
     <row r="6">
@@ -27504,16 +27609,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>122.23</v>
+        <v>124.31</v>
       </c>
       <c r="D6" t="n">
-        <v>1.977306858001016</v>
+        <v>1.701709891188741</v>
       </c>
       <c r="E6" t="n">
-        <v>22.31805634064645</v>
+        <v>22.40688250729537</v>
       </c>
       <c r="F6" t="n">
-        <v>13.00830076571879</v>
+        <v>14.93137419771335</v>
       </c>
     </row>
     <row r="7">
@@ -27528,16 +27633,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>130.98</v>
+        <v>145.05</v>
       </c>
       <c r="D7" t="n">
-        <v>1.166293349810754</v>
+        <v>10.74209803023365</v>
       </c>
       <c r="E7" t="n">
-        <v>33.61899840132232</v>
+        <v>43.89126368322292</v>
       </c>
       <c r="F7" t="n">
-        <v>24.11306746232529</v>
+        <v>37.44541483745827</v>
       </c>
     </row>
     <row r="8">
@@ -27552,16 +27657,16 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>130.31</v>
+        <v>133.69</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.04602285801948991</v>
+        <v>2.593814749443624</v>
       </c>
       <c r="E8" t="n">
-        <v>31.15206356846376</v>
+        <v>30.83239164895124</v>
       </c>
       <c r="F8" t="n">
-        <v>20.06630393925242</v>
+        <v>23.18060143994056</v>
       </c>
     </row>
     <row r="9">
@@ -27576,16 +27681,16 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>122.72</v>
+        <v>125.22</v>
       </c>
       <c r="D9" t="n">
-        <v>1.867684900805178</v>
+        <v>2.037157757496733</v>
       </c>
       <c r="E9" t="n">
-        <v>25.56608020896913</v>
+        <v>23.96797719523978</v>
       </c>
       <c r="F9" t="n">
-        <v>13.352297050706</v>
+        <v>15.66146216337521</v>
       </c>
     </row>
     <row r="10">
@@ -27600,16 +27705,16 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>124.65</v>
+        <v>126.2</v>
       </c>
       <c r="D10" t="n">
-        <v>0.9965969859017987</v>
+        <v>1.243481748896902</v>
       </c>
       <c r="E10" t="n">
-        <v>25.38865879601126</v>
+        <v>23.35550153845947</v>
       </c>
       <c r="F10" t="n">
-        <v>14.80696792476981</v>
+        <v>16.23457161737625</v>
       </c>
     </row>
     <row r="11">
@@ -27624,16 +27729,16 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>139.77</v>
+        <v>141.62</v>
       </c>
       <c r="D11" t="n">
-        <v>1.717487810203044</v>
+        <v>1.323603062173562</v>
       </c>
       <c r="E11" t="n">
-        <v>46.09946350731025</v>
+        <v>44.18197132280049</v>
       </c>
       <c r="F11" t="n">
-        <v>17.66345925047919</v>
+        <v>19.22085640017788</v>
       </c>
     </row>
     <row r="12">
@@ -27648,16 +27753,16 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>130.72</v>
+        <v>133.7</v>
       </c>
       <c r="D12" t="n">
-        <v>2.109045461646608</v>
+        <v>2.279681762545893</v>
       </c>
       <c r="E12" t="n">
-        <v>31.60603899994874</v>
+        <v>31.65071076529042</v>
       </c>
       <c r="F12" t="n">
-        <v>18.56064368117501</v>
+        <v>21.26344905273177</v>
       </c>
     </row>
     <row r="13">
@@ -27672,16 +27777,16 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>129.17</v>
+        <v>130.47</v>
       </c>
       <c r="D13" t="n">
-        <v>1.056172742919737</v>
+        <v>1.006425640628628</v>
       </c>
       <c r="E13" t="n">
-        <v>28.07046898245202</v>
+        <v>25.64466844969539</v>
       </c>
       <c r="F13" t="n">
-        <v>26.45609032403999</v>
+        <v>27.72877684119763</v>
       </c>
     </row>
     <row r="14">
@@ -27696,16 +27801,16 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>122.11</v>
+        <v>123.47</v>
       </c>
       <c r="D14" t="n">
-        <v>1.042614811750098</v>
+        <v>1.113749897633287</v>
       </c>
       <c r="E14" t="n">
-        <v>22.71116817298007</v>
+        <v>21.73888482986941</v>
       </c>
       <c r="F14" t="n">
-        <v>11.54462694544249</v>
+        <v>12.78695511386278</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Otomatik veri güncelleme (03.09.2026 15:12 UTC)
</commit_message>
<xml_diff>
--- a/enflasyon/enflasyon.xlsx
+++ b/enflasyon/enflasyon.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E260"/>
+  <dimension ref="A1:E261"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4801,6 +4801,23 @@
       </c>
       <c r="E260" t="n">
         <v>19.86016871927905</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B261" t="n">
+        <v>134.75</v>
+      </c>
+      <c r="C261" t="n">
+        <v>1.844153881036958</v>
+      </c>
+      <c r="D261" t="n">
+        <v>31.50734282091285</v>
+      </c>
+      <c r="E261" t="n">
+        <v>22.07057467253308</v>
       </c>
     </row>
   </sheetData>
@@ -4814,7 +4831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N260"/>
+  <dimension ref="A1:N261"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16283,6 +16300,50 @@
       </c>
       <c r="N260" t="n">
         <v>123.47</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B261" t="n">
+        <v>134.31</v>
+      </c>
+      <c r="C261" t="n">
+        <v>139.12</v>
+      </c>
+      <c r="D261" t="n">
+        <v>107.77</v>
+      </c>
+      <c r="E261" t="n">
+        <v>148.08</v>
+      </c>
+      <c r="F261" t="n">
+        <v>126.49</v>
+      </c>
+      <c r="G261" t="n">
+        <v>146.07</v>
+      </c>
+      <c r="H261" t="n">
+        <v>140.14</v>
+      </c>
+      <c r="I261" t="n">
+        <v>128.48</v>
+      </c>
+      <c r="J261" t="n">
+        <v>128.56</v>
+      </c>
+      <c r="K261" t="n">
+        <v>153.83</v>
+      </c>
+      <c r="L261" t="n">
+        <v>135.7</v>
+      </c>
+      <c r="M261" t="n">
+        <v>130.54</v>
+      </c>
+      <c r="N261" t="n">
+        <v>126.42</v>
       </c>
     </row>
   </sheetData>
@@ -16296,7 +16357,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N260"/>
+  <dimension ref="A1:N261"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27453,6 +27514,50 @@
       </c>
       <c r="N260" t="n">
         <v>21.73888482986941</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B261" t="n">
+        <v>33.78988040090669</v>
+      </c>
+      <c r="C261" t="n">
+        <v>30.42224822913602</v>
+      </c>
+      <c r="D261" t="n">
+        <v>13.15707827013983</v>
+      </c>
+      <c r="E261" t="n">
+        <v>39.77455728429897</v>
+      </c>
+      <c r="F261" t="n">
+        <v>23.5763577628787</v>
+      </c>
+      <c r="G261" t="n">
+        <v>43.45661506527607</v>
+      </c>
+      <c r="H261" t="n">
+        <v>35.07642610694981</v>
+      </c>
+      <c r="I261" t="n">
+        <v>25.66465697868268</v>
+      </c>
+      <c r="J261" t="n">
+        <v>23.42910595461436</v>
+      </c>
+      <c r="K261" t="n">
+        <v>53.44298409541148</v>
+      </c>
+      <c r="L261" t="n">
+        <v>31.1578146221104</v>
+      </c>
+      <c r="M261" t="n">
+        <v>25.07890495260689</v>
+      </c>
+      <c r="N261" t="n">
+        <v>23.64687142352469</v>
       </c>
     </row>
   </sheetData>
@@ -27513,16 +27618,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>134.02</v>
+        <v>134.31</v>
       </c>
       <c r="D2" t="n">
-        <v>1.614982182121483</v>
+        <v>0.2163856140874332</v>
       </c>
       <c r="E2" t="n">
-        <v>37.53005127954092</v>
+        <v>33.78988040090669</v>
       </c>
       <c r="F2" t="n">
-        <v>21.82652154856619</v>
+        <v>22.09013661534045</v>
       </c>
     </row>
     <row r="3">
@@ -27537,16 +27642,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>130.15</v>
+        <v>139.12</v>
       </c>
       <c r="D3" t="n">
-        <v>1.934523809523814</v>
+        <v>6.892047637341525</v>
       </c>
       <c r="E3" t="n">
-        <v>29.38189201377268</v>
+        <v>30.42224822913602</v>
       </c>
       <c r="F3" t="n">
-        <v>16.2868521420896</v>
+        <v>24.30139738768733</v>
       </c>
     </row>
     <row r="4">
@@ -27561,16 +27666,16 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>111.73</v>
+        <v>107.77</v>
       </c>
       <c r="D4" t="n">
-        <v>-3.929492691315561</v>
+        <v>-3.544258480264928</v>
       </c>
       <c r="E4" t="n">
-        <v>16.47854628756089</v>
+        <v>13.15707827013983</v>
       </c>
       <c r="F4" t="n">
-        <v>2.758604569261713</v>
+        <v>-0.8834259873862438</v>
       </c>
     </row>
     <row r="5">
@@ -27585,16 +27690,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>144.81</v>
+        <v>148.08</v>
       </c>
       <c r="D5" t="n">
-        <v>2.252506708092072</v>
+        <v>2.25813134452042</v>
       </c>
       <c r="E5" t="n">
-        <v>40.32266749804405</v>
+        <v>39.77455728429897</v>
       </c>
       <c r="F5" t="n">
-        <v>25.91930196781995</v>
+        <v>28.76272519435659</v>
       </c>
     </row>
     <row r="6">
@@ -27609,16 +27714,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>124.31</v>
+        <v>126.49</v>
       </c>
       <c r="D6" t="n">
-        <v>1.701709891188741</v>
+        <v>1.753680315340667</v>
       </c>
       <c r="E6" t="n">
-        <v>22.40688250729537</v>
+        <v>23.5763577628787</v>
       </c>
       <c r="F6" t="n">
-        <v>14.93137419771335</v>
+        <v>16.94690308316918</v>
       </c>
     </row>
     <row r="7">
@@ -27633,16 +27738,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>145.05</v>
+        <v>146.07</v>
       </c>
       <c r="D7" t="n">
-        <v>10.74209803023365</v>
+        <v>0.7032057911064982</v>
       </c>
       <c r="E7" t="n">
-        <v>43.89126368322292</v>
+        <v>43.45661506527607</v>
       </c>
       <c r="F7" t="n">
-        <v>37.44541483745827</v>
+        <v>38.41193895420565</v>
       </c>
     </row>
     <row r="8">
@@ -27657,16 +27762,16 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>133.69</v>
+        <v>140.14</v>
       </c>
       <c r="D8" t="n">
-        <v>2.593814749443624</v>
+        <v>4.824594210486932</v>
       </c>
       <c r="E8" t="n">
-        <v>30.83239164895124</v>
+        <v>35.07642610694981</v>
       </c>
       <c r="F8" t="n">
-        <v>23.18060143994056</v>
+        <v>29.12356560545493</v>
       </c>
     </row>
     <row r="9">
@@ -27681,16 +27786,16 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>125.22</v>
+        <v>128.48</v>
       </c>
       <c r="D9" t="n">
-        <v>2.037157757496733</v>
+        <v>2.603417984347534</v>
       </c>
       <c r="E9" t="n">
-        <v>23.96797719523978</v>
+        <v>25.66465697868268</v>
       </c>
       <c r="F9" t="n">
-        <v>15.66146216337521</v>
+        <v>18.67261347029583</v>
       </c>
     </row>
     <row r="10">
@@ -27705,16 +27810,16 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>126.2</v>
+        <v>128.56</v>
       </c>
       <c r="D10" t="n">
-        <v>1.243481748896902</v>
+        <v>1.870047543581621</v>
       </c>
       <c r="E10" t="n">
-        <v>23.35550153845947</v>
+        <v>23.42910595461436</v>
       </c>
       <c r="F10" t="n">
-        <v>16.23457161737625</v>
+        <v>18.4082133686996</v>
       </c>
     </row>
     <row r="11">
@@ -27729,16 +27834,16 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>141.62</v>
+        <v>153.83</v>
       </c>
       <c r="D11" t="n">
-        <v>1.323603062173562</v>
+        <v>8.621663606835206</v>
       </c>
       <c r="E11" t="n">
-        <v>44.18197132280049</v>
+        <v>53.44298409541148</v>
       </c>
       <c r="F11" t="n">
-        <v>19.22085640017788</v>
+        <v>29.49967758818928</v>
       </c>
     </row>
     <row r="12">
@@ -27753,16 +27858,16 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>133.7</v>
+        <v>135.7</v>
       </c>
       <c r="D12" t="n">
-        <v>2.279681762545893</v>
+        <v>1.495886312640238</v>
       </c>
       <c r="E12" t="n">
-        <v>31.65071076529042</v>
+        <v>31.1578146221104</v>
       </c>
       <c r="F12" t="n">
-        <v>21.26344905273177</v>
+        <v>23.07741238934704</v>
       </c>
     </row>
     <row r="13">
@@ -27777,16 +27882,16 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>130.47</v>
+        <v>130.54</v>
       </c>
       <c r="D13" t="n">
-        <v>1.006425640628628</v>
+        <v>0.05365218057791221</v>
       </c>
       <c r="E13" t="n">
-        <v>25.64466844969539</v>
+        <v>25.07890495260689</v>
       </c>
       <c r="F13" t="n">
-        <v>27.72877684119763</v>
+        <v>27.79730611519842</v>
       </c>
     </row>
     <row r="14">
@@ -27801,16 +27906,16 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>123.47</v>
+        <v>126.42</v>
       </c>
       <c r="D14" t="n">
-        <v>1.113749897633287</v>
+        <v>2.389244350854458</v>
       </c>
       <c r="E14" t="n">
-        <v>21.73888482986941</v>
+        <v>23.64687142352469</v>
       </c>
       <c r="F14" t="n">
-        <v>12.78695511386278</v>
+        <v>15.48171106742151</v>
       </c>
     </row>
   </sheetData>

</xml_diff>